<commit_message>
Complete Day 34 batch report generation
</commit_message>
<xml_diff>
--- a/output/cashflow_intelligence.xlsx
+++ b/output/cashflow_intelligence.xlsx
@@ -485,26 +485,26 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>3.35</v>
+        <v>0.9</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>High Quality</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>81.48999999999999</v>
+        <v>6.86</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Capital Intensive</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>61.49</v>
+        <v>37.19</v>
       </c>
       <c r="H2" t="n">
-        <v>70.78</v>
+        <v>51.52</v>
       </c>
       <c r="I2" t="b">
         <v>0</v>
@@ -925,7 +925,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.87</v>
+        <v>0.71</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -941,7 +941,7 @@
         </is>
       </c>
       <c r="G12" t="n">
-        <v>9.73</v>
+        <v>3.67</v>
       </c>
       <c r="H12" t="n">
         <v>70.94</v>

</xml_diff>